<commit_message>
Backfill del histórico: ruedas del 30 y 31 de julio
El job diario venía clavado por la referencia vencida (S31L6), así que esas dos
ruedas nunca se escribieron. Se traen de 1816 (precioDirty) para todo el universo
del fork: 157 precios por fecha sobre 188 columnas; los 31 restantes son
instrumentos ya vencidos o sin mapeo a 1816.

No se usó el historicos del repo del colega porque sólo cubre 78 tickers y
hubiera perdido las columnas de ONs y subsoberanos.

Verificado: sin descartes de la guarda de escala y sin saltos day-over-day
mayores al 15% en la muestra de control.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -15,8 +15,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd\-mm\-yy;@"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -47,9 +49,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -415,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:GG49"/>
+  <dimension ref="A1:GG51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="10.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -23473,6 +23476,958 @@
         <v>100.75</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>46233</v>
+      </c>
+      <c r="G50" t="n">
+        <v>107.089</v>
+      </c>
+      <c r="H50" t="n">
+        <v>124.55</v>
+      </c>
+      <c r="I50" t="n">
+        <v>112.85</v>
+      </c>
+      <c r="J50" t="n">
+        <v>127.5</v>
+      </c>
+      <c r="K50" t="n">
+        <v>119.75</v>
+      </c>
+      <c r="L50" t="n">
+        <v>143.7</v>
+      </c>
+      <c r="M50" t="n">
+        <v>131.1</v>
+      </c>
+      <c r="N50" t="n">
+        <v>123.7</v>
+      </c>
+      <c r="O50" t="n">
+        <v>125.25</v>
+      </c>
+      <c r="P50" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>112.6</v>
+      </c>
+      <c r="S50" t="n">
+        <v>167.2</v>
+      </c>
+      <c r="T50" t="n">
+        <v>294.05</v>
+      </c>
+      <c r="U50" t="n">
+        <v>217.15</v>
+      </c>
+      <c r="V50" t="n">
+        <v>120.55</v>
+      </c>
+      <c r="W50" t="n">
+        <v>387.4</v>
+      </c>
+      <c r="X50" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="Y50" t="n">
+        <v>271</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>98</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>345.55</v>
+      </c>
+      <c r="AB50" t="n">
+        <v>93.98</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>89.2</v>
+      </c>
+      <c r="AD50" t="n">
+        <v>127.15</v>
+      </c>
+      <c r="AE50" t="n">
+        <v>118.05</v>
+      </c>
+      <c r="AF50" t="n">
+        <v>112.25</v>
+      </c>
+      <c r="AG50" t="n">
+        <v>106.85</v>
+      </c>
+      <c r="AH50" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="AJ50" t="n">
+        <v>147400</v>
+      </c>
+      <c r="AK50" t="n">
+        <v>146300</v>
+      </c>
+      <c r="AL50" t="n">
+        <v>125700</v>
+      </c>
+      <c r="AM50" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="AN50" t="n">
+        <v>97</v>
+      </c>
+      <c r="AO50" t="n">
+        <v>54.89999999999998</v>
+      </c>
+      <c r="AP50" t="n">
+        <v>96.88999999999999</v>
+      </c>
+      <c r="AQ50" t="n">
+        <v>56.35</v>
+      </c>
+      <c r="AR50" t="n">
+        <v>79.12</v>
+      </c>
+      <c r="AS50" t="n">
+        <v>81.73999999999999</v>
+      </c>
+      <c r="AT50" t="n">
+        <v>74.89</v>
+      </c>
+      <c r="AU50" t="n">
+        <v>55.63</v>
+      </c>
+      <c r="AV50" t="n">
+        <v>57.45</v>
+      </c>
+      <c r="AW50" t="n">
+        <v>81.81999999999999</v>
+      </c>
+      <c r="AX50" t="n">
+        <v>85.81999999999999</v>
+      </c>
+      <c r="AY50" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="AZ50" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="BA50" t="n">
+        <v>102.65</v>
+      </c>
+      <c r="BB50" t="n">
+        <v>103</v>
+      </c>
+      <c r="BC50" t="n">
+        <v>92.80000000000001</v>
+      </c>
+      <c r="BD50" t="n">
+        <v>92.51000000000001</v>
+      </c>
+      <c r="BE50" t="n">
+        <v>97.2</v>
+      </c>
+      <c r="BF50" t="n">
+        <v>90.40000000000001</v>
+      </c>
+      <c r="BH50" t="n">
+        <v>164.9</v>
+      </c>
+      <c r="BI50" t="n">
+        <v>104.06</v>
+      </c>
+      <c r="BK50" t="n">
+        <v>144990</v>
+      </c>
+      <c r="BM50" t="n">
+        <v>100.95</v>
+      </c>
+      <c r="BN50" t="n">
+        <v>105.45</v>
+      </c>
+      <c r="BO50" t="n">
+        <v>113.3</v>
+      </c>
+      <c r="BP50" t="n">
+        <v>107.9</v>
+      </c>
+      <c r="BQ50" t="n">
+        <v>147500</v>
+      </c>
+      <c r="BR50" t="n">
+        <v>120000</v>
+      </c>
+      <c r="BS50" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="BT50" t="n">
+        <v>84.48999999999999</v>
+      </c>
+      <c r="BU50" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="BV50" t="n">
+        <v>102.28</v>
+      </c>
+      <c r="BW50" t="n">
+        <v>94</v>
+      </c>
+      <c r="BX50" t="n">
+        <v>84.25</v>
+      </c>
+      <c r="BY50" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="CA50" t="n">
+        <v>94.28999999999999</v>
+      </c>
+      <c r="CB50" t="n">
+        <v>117.65</v>
+      </c>
+      <c r="CC50" t="n">
+        <v>121.12</v>
+      </c>
+      <c r="CE50" t="n">
+        <v>112.6</v>
+      </c>
+      <c r="CF50" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="CG50" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="CS50" t="n">
+        <v>47.99999999999999</v>
+      </c>
+      <c r="CV50" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="CX50" t="n">
+        <v>111.95</v>
+      </c>
+      <c r="CY50" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="DA50" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="DB50" t="n">
+        <v>108.25</v>
+      </c>
+      <c r="DD50" t="n">
+        <v>104</v>
+      </c>
+      <c r="DE50" t="n">
+        <v>79.47</v>
+      </c>
+      <c r="DF50" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="DH50" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="DI50" t="n">
+        <v>108.05</v>
+      </c>
+      <c r="DJ50" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="DK50" t="n">
+        <v>109.9</v>
+      </c>
+      <c r="DL50" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="DM50" t="n">
+        <v>84.19</v>
+      </c>
+      <c r="DN50" t="n">
+        <v>51.25999999999999</v>
+      </c>
+      <c r="DO50" t="n">
+        <v>111</v>
+      </c>
+      <c r="DP50" t="n">
+        <v>108.5</v>
+      </c>
+      <c r="DQ50" t="n">
+        <v>103.65</v>
+      </c>
+      <c r="DR50" t="n">
+        <v>111.65</v>
+      </c>
+      <c r="DS50" t="n">
+        <v>109.25</v>
+      </c>
+      <c r="DT50" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="DU50" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="DV50" t="n">
+        <v>108.9</v>
+      </c>
+      <c r="DW50" t="n">
+        <v>111.25</v>
+      </c>
+      <c r="DX50" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="DY50" t="n">
+        <v>108.7</v>
+      </c>
+      <c r="DZ50" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="EA50" t="n">
+        <v>108.65</v>
+      </c>
+      <c r="EB50" t="n">
+        <v>110.4</v>
+      </c>
+      <c r="EC50" t="n">
+        <v>108.45</v>
+      </c>
+      <c r="ED50" t="n">
+        <v>111.65</v>
+      </c>
+      <c r="EE50" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="EF50" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="EG50" t="n">
+        <v>92.60999999999999</v>
+      </c>
+      <c r="EH50" t="n">
+        <v>114.15</v>
+      </c>
+      <c r="EI50" t="n">
+        <v>107.85</v>
+      </c>
+      <c r="EJ50" t="n">
+        <v>110.05</v>
+      </c>
+      <c r="EK50" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="EL50" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="EM50" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="EN50" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="EO50" t="n">
+        <v>109.65</v>
+      </c>
+      <c r="EP50" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="EQ50" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="ER50" t="n">
+        <v>108.15</v>
+      </c>
+      <c r="ES50" t="n">
+        <v>110.45</v>
+      </c>
+      <c r="ET50" t="n">
+        <v>103.55</v>
+      </c>
+      <c r="EU50" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="EV50" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="EW50" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="EX50" t="n">
+        <v>108.55</v>
+      </c>
+      <c r="EY50" t="n">
+        <v>111.2</v>
+      </c>
+      <c r="EZ50" t="n">
+        <v>105.65</v>
+      </c>
+      <c r="FA50" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="FB50" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="FC50" t="n">
+        <v>106</v>
+      </c>
+      <c r="FD50" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="FE50" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="FF50" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="FG50" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="FH50" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="FI50" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="FJ50" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="FK50" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="FL50" t="n">
+        <v>104</v>
+      </c>
+      <c r="FM50" t="n">
+        <v>101</v>
+      </c>
+      <c r="FN50" t="n">
+        <v>101</v>
+      </c>
+      <c r="FO50" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="FP50" t="n">
+        <v>109.8</v>
+      </c>
+      <c r="FQ50" t="n">
+        <v>102.15</v>
+      </c>
+      <c r="FR50" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="FS50" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="FT50" t="n">
+        <v>110.45</v>
+      </c>
+      <c r="FU50" t="n">
+        <v>100</v>
+      </c>
+      <c r="FV50" t="n">
+        <v>106.45</v>
+      </c>
+      <c r="FW50" t="n">
+        <v>103.45</v>
+      </c>
+      <c r="FX50" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="FY50" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="FZ50" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="GA50" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GB50" t="n">
+        <v>102.55</v>
+      </c>
+      <c r="GC50" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="GD50" t="n">
+        <v>104.65</v>
+      </c>
+      <c r="GE50" t="n">
+        <v>103.75</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>46234</v>
+      </c>
+      <c r="G51" t="n">
+        <v>107.27</v>
+      </c>
+      <c r="H51" t="n">
+        <v>124.801</v>
+      </c>
+      <c r="I51" t="n">
+        <v>113.1</v>
+      </c>
+      <c r="J51" t="n">
+        <v>127.801</v>
+      </c>
+      <c r="K51" t="n">
+        <v>119.89</v>
+      </c>
+      <c r="L51" t="n">
+        <v>144.5</v>
+      </c>
+      <c r="M51" t="n">
+        <v>131.1</v>
+      </c>
+      <c r="N51" t="n">
+        <v>123.59</v>
+      </c>
+      <c r="O51" t="n">
+        <v>125.44</v>
+      </c>
+      <c r="P51" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>113</v>
+      </c>
+      <c r="S51" t="n">
+        <v>167.45</v>
+      </c>
+      <c r="T51" t="n">
+        <v>294.7</v>
+      </c>
+      <c r="U51" t="n">
+        <v>217.45</v>
+      </c>
+      <c r="V51" t="n">
+        <v>121</v>
+      </c>
+      <c r="W51" t="n">
+        <v>387.5</v>
+      </c>
+      <c r="X51" t="n">
+        <v>104.15</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>271.4</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="AA51" t="n">
+        <v>347</v>
+      </c>
+      <c r="AB51" t="n">
+        <v>94.19</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>89.8</v>
+      </c>
+      <c r="AD51" t="n">
+        <v>127.399</v>
+      </c>
+      <c r="AE51" t="n">
+        <v>117.9</v>
+      </c>
+      <c r="AF51" t="n">
+        <v>112.75</v>
+      </c>
+      <c r="AG51" t="n">
+        <v>107.25</v>
+      </c>
+      <c r="AH51" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="AJ51" t="n">
+        <v>147730</v>
+      </c>
+      <c r="AK51" t="n">
+        <v>146750</v>
+      </c>
+      <c r="AL51" t="n">
+        <v>126000</v>
+      </c>
+      <c r="AM51" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="AN51" t="n">
+        <v>96.75</v>
+      </c>
+      <c r="AO51" t="n">
+        <v>55.13</v>
+      </c>
+      <c r="AP51" t="n">
+        <v>96.84999999999999</v>
+      </c>
+      <c r="AQ51" t="n">
+        <v>56.60000000000001</v>
+      </c>
+      <c r="AR51" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="AS51" t="n">
+        <v>82.39</v>
+      </c>
+      <c r="AT51" t="n">
+        <v>74.8</v>
+      </c>
+      <c r="AU51" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="AV51" t="n">
+        <v>58.09999999999999</v>
+      </c>
+      <c r="AW51" t="n">
+        <v>82.59</v>
+      </c>
+      <c r="AX51" t="n">
+        <v>86.19</v>
+      </c>
+      <c r="AY51" t="n">
+        <v>77.36</v>
+      </c>
+      <c r="AZ51" t="n">
+        <v>70.64</v>
+      </c>
+      <c r="BA51" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="BB51" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="BC51" t="n">
+        <v>92.90000000000001</v>
+      </c>
+      <c r="BD51" t="n">
+        <v>92.99000000000001</v>
+      </c>
+      <c r="BE51" t="n">
+        <v>97.03</v>
+      </c>
+      <c r="BF51" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="BH51" t="n">
+        <v>165.1</v>
+      </c>
+      <c r="BI51" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="BK51" t="n">
+        <v>145500</v>
+      </c>
+      <c r="BM51" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="BN51" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="BO51" t="n">
+        <v>113.85</v>
+      </c>
+      <c r="BP51" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="BQ51" t="n">
+        <v>148000</v>
+      </c>
+      <c r="BR51" t="n">
+        <v>119800</v>
+      </c>
+      <c r="BS51" t="n">
+        <v>91.45</v>
+      </c>
+      <c r="BT51" t="n">
+        <v>84.55</v>
+      </c>
+      <c r="BU51" t="n">
+        <v>81.72</v>
+      </c>
+      <c r="BV51" t="n">
+        <v>102.399</v>
+      </c>
+      <c r="BW51" t="n">
+        <v>96.73999999999999</v>
+      </c>
+      <c r="BX51" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="BY51" t="n">
+        <v>104</v>
+      </c>
+      <c r="CA51" t="n">
+        <v>94.55</v>
+      </c>
+      <c r="CB51" t="n">
+        <v>117.1</v>
+      </c>
+      <c r="CC51" t="n">
+        <v>121.4</v>
+      </c>
+      <c r="CE51" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="CF51" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="CG51" t="n">
+        <v>102.65</v>
+      </c>
+      <c r="CS51" t="n">
+        <v>49.00000000000001</v>
+      </c>
+      <c r="CV51" t="n">
+        <v>64.45</v>
+      </c>
+      <c r="CX51" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="DA51" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="DB51" t="n">
+        <v>104</v>
+      </c>
+      <c r="DD51" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="DE51" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="DF51" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="DH51" t="n">
+        <v>109.25</v>
+      </c>
+      <c r="DI51" t="n">
+        <v>108.7</v>
+      </c>
+      <c r="DJ51" t="n">
+        <v>108.25</v>
+      </c>
+      <c r="DK51" t="n">
+        <v>109.65</v>
+      </c>
+      <c r="DL51" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="DM51" t="n">
+        <v>84.02</v>
+      </c>
+      <c r="DN51" t="n">
+        <v>51.46000000000001</v>
+      </c>
+      <c r="DO51" t="n">
+        <v>110.85</v>
+      </c>
+      <c r="DP51" t="n">
+        <v>107.9</v>
+      </c>
+      <c r="DQ51" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="DR51" t="n">
+        <v>112</v>
+      </c>
+      <c r="DS51" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="DT51" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="DU51" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="DV51" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="DW51" t="n">
+        <v>112</v>
+      </c>
+      <c r="DX51" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="DY51" t="n">
+        <v>108.8</v>
+      </c>
+      <c r="DZ51" t="n">
+        <v>113</v>
+      </c>
+      <c r="EA51" t="n">
+        <v>109.35</v>
+      </c>
+      <c r="EB51" t="n">
+        <v>110.4</v>
+      </c>
+      <c r="EC51" t="n">
+        <v>108.9</v>
+      </c>
+      <c r="ED51" t="n">
+        <v>111.55</v>
+      </c>
+      <c r="EE51" t="n">
+        <v>108.7</v>
+      </c>
+      <c r="EF51" t="n">
+        <v>110</v>
+      </c>
+      <c r="EG51" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="EH51" t="n">
+        <v>114.45</v>
+      </c>
+      <c r="EI51" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="EJ51" t="n">
+        <v>110.6</v>
+      </c>
+      <c r="EK51" t="n">
+        <v>111</v>
+      </c>
+      <c r="EL51" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="EM51" t="n">
+        <v>107</v>
+      </c>
+      <c r="EN51" t="n">
+        <v>107.9</v>
+      </c>
+      <c r="EO51" t="n">
+        <v>109</v>
+      </c>
+      <c r="EP51" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="EQ51" t="n">
+        <v>108.75</v>
+      </c>
+      <c r="ER51" t="n">
+        <v>108.55</v>
+      </c>
+      <c r="ES51" t="n">
+        <v>109.9</v>
+      </c>
+      <c r="ET51" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="EU51" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="EV51" t="n">
+        <v>103.65</v>
+      </c>
+      <c r="EW51" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="EX51" t="n">
+        <v>108.2</v>
+      </c>
+      <c r="EY51" t="n">
+        <v>111.1</v>
+      </c>
+      <c r="EZ51" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="FA51" t="n">
+        <v>104</v>
+      </c>
+      <c r="FB51" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="FC51" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="FD51" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="FE51" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="FF51" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="FG51" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="FH51" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="FI51" t="n">
+        <v>104</v>
+      </c>
+      <c r="FJ51" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="FK51" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="FL51" t="n">
+        <v>104</v>
+      </c>
+      <c r="FM51" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="FN51" t="n">
+        <v>104</v>
+      </c>
+      <c r="FO51" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="FP51" t="n">
+        <v>110.75</v>
+      </c>
+      <c r="FQ51" t="n">
+        <v>102.15</v>
+      </c>
+      <c r="FR51" t="n">
+        <v>103</v>
+      </c>
+      <c r="FS51" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="FT51" t="n">
+        <v>110.25</v>
+      </c>
+      <c r="FU51" t="n">
+        <v>100</v>
+      </c>
+      <c r="FV51" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="FW51" t="n">
+        <v>104</v>
+      </c>
+      <c r="FX51" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="FY51" t="n">
+        <v>105.85</v>
+      </c>
+      <c r="FZ51" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="GA51" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="GB51" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GC51" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="GD51" t="n">
+        <v>104</v>
+      </c>
+      <c r="GE51" t="n">
+        <v>106.95</v>
+      </c>
+      <c r="GG51" t="n">
+        <v>100.6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>